<commit_message>
Tuned PID values for potential motor
</commit_message>
<xml_diff>
--- a/software/matlab/motors.xlsx
+++ b/software/matlab/motors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flipa\OneDrive - UBC\University\Course Materials\3rd year\ELEC 391\robot-piano-player\software\matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE98FAFC-BC9C-4594-BD43-79E9E9F2F8E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADFBBC3-55B0-4656-A966-0DEE3DB85C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A00A6A0-CC9E-4CD9-B7FE-C8C2B9679AFB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Motor</t>
   </si>
@@ -69,16 +69,41 @@
   </si>
   <si>
     <t>Maxon_ECi40</t>
+  </si>
+  <si>
+    <t>https://ca.robotshop.com/products/e-s-motor-60d-brushed-planetary-gear-motor-with-encoder-24v-800rpm?qd=67fa275660c08a525e76e18f421eb9a9</t>
+  </si>
+  <si>
+    <t>https://ca.robotshop.com/products/e-s-motor-60d-brushed-planetary-gear-motor-with-encoder-24v-2820rpm?qd=67fa275660c08a525e76e18f421eb9a9</t>
+  </si>
+  <si>
+    <t>https://ca.robotshop.com/products/e-s-motor-555-size-dc-motor-with-encoder-24v-16000-rpm?qd=5f2b900c5da47b37b4e2bfa7d58352d4</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>60PG-997-4.25-EN</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="170" formatCode="0.0"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -104,8 +129,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,7 +467,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A19DF-95F4-4146-B9C9-3E67B92D887F}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" customWidth="1"/>
@@ -448,7 +475,7 @@
     <col min="6" max="6" width="11.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -470,8 +497,11 @@
       <c r="G1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -494,7 +524,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -517,7 +547,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -540,7 +570,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>10</v>
       </c>
@@ -561,6 +591,45 @@
       </c>
       <c r="G5">
         <v>496</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7">
+        <f>24/20</f>
+        <v>1.2</v>
+      </c>
+      <c r="C7" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D7" s="1">
+        <f>0.5/24*1000</f>
+        <v>20.833333333333332</v>
+      </c>
+      <c r="E7" s="2">
+        <f>MAX(E2:E5)*1.2</f>
+        <v>3672</v>
+      </c>
+      <c r="F7">
+        <v>12000</v>
+      </c>
+      <c r="G7">
+        <v>1600</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="H8" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tuned PID parameters taking into account gear system of motor, added simulink model
</commit_message>
<xml_diff>
--- a/software/matlab/motors.xlsx
+++ b/software/matlab/motors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flipa\OneDrive - UBC\University\Course Materials\3rd year\ELEC 391\robot-piano-player\software\matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADFBBC3-55B0-4656-A966-0DEE3DB85C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92242AF5-3EF4-46E3-9698-F047D90BF24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A00A6A0-CC9E-4CD9-B7FE-C8C2B9679AFB}"/>
   </bookViews>
@@ -91,9 +91,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -104,6 +104,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -126,15 +134,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -610,8 +621,8 @@
         <v>0.2</v>
       </c>
       <c r="D7" s="1">
-        <f>0.5/24*1000</f>
-        <v>20.833333333333332</v>
+        <f>1.62/12*1000</f>
+        <v>135</v>
       </c>
       <c r="E7" s="2">
         <f>MAX(E2:E5)*1.2</f>
@@ -623,7 +634,7 @@
       <c r="G7">
         <v>1600</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -633,7 +644,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H7" r:id="rId1" xr:uid="{A8D4DA74-31D2-4D8D-ABB1-19E58F228A4D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="256" orientation="landscape" horizontalDpi="500" verticalDpi="500" copies="0" r:id="rId1"/>
+  <pageSetup paperSize="256" orientation="landscape" horizontalDpi="500" verticalDpi="500" copies="0" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Accounting for gear ratio, reducing estimate of rotor inertia
</commit_message>
<xml_diff>
--- a/software/matlab/motors.xlsx
+++ b/software/matlab/motors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flipa\OneDrive - UBC\University\Course Materials\3rd year\ELEC 391\robot-piano-player\software\matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92242AF5-3EF4-46E3-9698-F047D90BF24B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9D94DC-CEB1-429C-B220-2F81DF34BC08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A00A6A0-CC9E-4CD9-B7FE-C8C2B9679AFB}"/>
   </bookViews>
@@ -621,12 +621,11 @@
         <v>0.2</v>
       </c>
       <c r="D7" s="1">
-        <f>1.62/12*1000</f>
-        <v>135</v>
+        <f>0.5/12*1000</f>
+        <v>41.666666666666664</v>
       </c>
       <c r="E7" s="2">
-        <f>MAX(E2:E5)*1.2</f>
-        <v>3672</v>
+        <v>2200</v>
       </c>
       <c r="F7">
         <v>12000</v>

</xml_diff>

<commit_message>
Added S curve ramp up and tuned PID to approximate stepper motor driver
</commit_message>
<xml_diff>
--- a/software/matlab/motors.xlsx
+++ b/software/matlab/motors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flipa\OneDrive - UBC\University\Course Materials\3rd year\ELEC 391\robot-piano-player\software\matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9D94DC-CEB1-429C-B220-2F81DF34BC08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D2D0F9-3948-4902-A3AA-CD0E783363AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A00A6A0-CC9E-4CD9-B7FE-C8C2B9679AFB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Motor</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>60PG-997-4.25-EN</t>
+  </si>
+  <si>
+    <t>https://datasheet4u.com/pdf-down/N/E/M/NEMA17-Servotronix.pdf</t>
+  </si>
+  <si>
+    <t>NEMA17S</t>
   </si>
 </sst>
 </file>
@@ -478,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A19DF-95F4-4146-B9C9-3E67B92D887F}">
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" customWidth="1"/>
@@ -621,8 +627,8 @@
         <v>0.2</v>
       </c>
       <c r="D7" s="1">
-        <f>0.5/12*1000</f>
-        <v>41.666666666666664</v>
+        <f>0.3/12*1000</f>
+        <v>24.999999999999996</v>
       </c>
       <c r="E7" s="2">
         <v>2200</v>
@@ -640,6 +646,35 @@
     <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="H8" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9">
+        <f>6/(1.8^2)</f>
+        <v>1.8518518518518516</v>
+      </c>
+      <c r="C9">
+        <f>C5</f>
+        <v>0.128</v>
+      </c>
+      <c r="D9">
+        <f>0.3/1.8*1000</f>
+        <v>166.66666666666666</v>
+      </c>
+      <c r="E9">
+        <v>57</v>
+      </c>
+      <c r="F9">
+        <v>12000</v>
+      </c>
+      <c r="G9">
+        <v>1600</v>
+      </c>
+      <c r="H9" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated motor parameter parsing, added gearbox inertia calculation, more detailed LTI simulations for current and speed
</commit_message>
<xml_diff>
--- a/software/matlab/motors.xlsx
+++ b/software/matlab/motors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flipa\OneDrive - UBC\University\Course Materials\3rd year\ELEC 391\robot-piano-player\software\matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4D2D0F9-3948-4902-A3AA-CD0E783363AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA4DC98-DF3F-4C99-9FD7-1732EF2C9F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A00A6A0-CC9E-4CD9-B7FE-C8C2B9679AFB}"/>
   </bookViews>
@@ -36,14 +36,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Motor</t>
   </si>
   <si>
-    <t>Maxon_EC90</t>
-  </si>
-  <si>
     <t>I_NL (mA)</t>
   </si>
   <si>
@@ -62,18 +59,6 @@
     <t>rpm_NL (rpm)</t>
   </si>
   <si>
-    <t>Maxon_RE65</t>
-  </si>
-  <si>
-    <t>Maxon_RE50</t>
-  </si>
-  <si>
-    <t>Maxon_ECi40</t>
-  </si>
-  <si>
-    <t>https://ca.robotshop.com/products/e-s-motor-60d-brushed-planetary-gear-motor-with-encoder-24v-800rpm?qd=67fa275660c08a525e76e18f421eb9a9</t>
-  </si>
-  <si>
     <t>https://ca.robotshop.com/products/e-s-motor-60d-brushed-planetary-gear-motor-with-encoder-24v-2820rpm?qd=67fa275660c08a525e76e18f421eb9a9</t>
   </si>
   <si>
@@ -86,10 +71,19 @@
     <t>60PG-997-4.25-EN</t>
   </si>
   <si>
-    <t>https://datasheet4u.com/pdf-down/N/E/M/NEMA17-Servotronix.pdf</t>
-  </si>
-  <si>
-    <t>NEMA17S</t>
+    <t>Gearbox Ratio</t>
+  </si>
+  <si>
+    <t>Stall Current (A)</t>
+  </si>
+  <si>
+    <t>RS555-EN</t>
+  </si>
+  <si>
+    <t>60PG-6055ZY</t>
+  </si>
+  <si>
+    <t>https://ca.robotshop.com/products/e-s-motor-60d-planetary-gear-motor-with-high-torque-and-compact-size-24v-1660rpm?qd=650ebc719b16f099bd5f5e09cc852c24</t>
   </si>
 </sst>
 </file>
@@ -99,7 +93,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,6 +116,25 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -131,7 +144,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -139,16 +152,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -484,204 +524,159 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A19DF-95F4-4146-B9C9-3E67B92D887F}">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.36328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.54296875" customWidth="1"/>
     <col min="6" max="6" width="11.81640625" customWidth="1"/>
+    <col min="7" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" ht="40" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
+      <c r="G1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="5">
+        <v>1.2</v>
+      </c>
+      <c r="C2" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="5">
+        <v>25</v>
+      </c>
+      <c r="E2" s="6">
+        <v>1471.4963</v>
+      </c>
+      <c r="F2" s="5">
+        <v>12000</v>
+      </c>
+      <c r="G2" s="5">
+        <v>1600</v>
+      </c>
+      <c r="H2" s="5">
+        <v>3.6</v>
+      </c>
+      <c r="I2" s="5">
+        <v>20</v>
+      </c>
+      <c r="J2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="G1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="3" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="5">
+        <v>3.692307692</v>
+      </c>
+      <c r="C3" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="D3" s="5">
+        <v>12.06972</v>
+      </c>
+      <c r="E3" s="6">
+        <v>192.24468999999999</v>
+      </c>
+      <c r="F3" s="5">
+        <v>16000</v>
+      </c>
+      <c r="G3" s="5">
+        <v>500</v>
+      </c>
+      <c r="H3" s="5">
+        <v>1</v>
+      </c>
+      <c r="I3" s="5">
+        <v>37</v>
+      </c>
+      <c r="J3" s="7" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
+      <c r="B4" s="5">
+        <v>1.6</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="D4" s="5">
+        <v>66.666666669999998</v>
+      </c>
+      <c r="E4" s="6">
+        <v>1434.6000899999999</v>
+      </c>
+      <c r="F4" s="5">
+        <v>6000</v>
+      </c>
+      <c r="G4" s="5">
+        <v>400</v>
+      </c>
+      <c r="H4" s="5">
+        <v>3.6</v>
+      </c>
+      <c r="I4" s="5">
+        <v>15</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>0.34300000000000003</v>
-      </c>
-      <c r="C2">
-        <v>0.26400000000000001</v>
-      </c>
-      <c r="D2">
-        <v>70.5</v>
-      </c>
-      <c r="E2">
-        <v>3060</v>
-      </c>
-      <c r="F2">
-        <v>3190</v>
-      </c>
-      <c r="G2">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3">
-        <v>8.2100000000000006E-2</v>
-      </c>
-      <c r="C3">
-        <v>3.1E-2</v>
-      </c>
-      <c r="D3">
-        <v>53.7</v>
-      </c>
-      <c r="E3">
-        <v>1290</v>
-      </c>
-      <c r="F3">
-        <v>4090</v>
-      </c>
-      <c r="G3">
-        <v>697</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
-        <v>0.10299999999999999</v>
-      </c>
-      <c r="C4">
-        <v>7.1999999999999995E-2</v>
-      </c>
-      <c r="D4">
-        <v>38.5</v>
-      </c>
-      <c r="E4">
-        <v>536</v>
-      </c>
-      <c r="F4">
-        <v>5950</v>
-      </c>
-      <c r="G4">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
-        <v>0.19500000000000001</v>
-      </c>
-      <c r="C5">
-        <v>0.128</v>
-      </c>
-      <c r="D5">
-        <v>36.4</v>
-      </c>
-      <c r="E5">
-        <v>78</v>
-      </c>
-      <c r="F5">
-        <v>4670</v>
-      </c>
-      <c r="G5">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="H6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7">
-        <f>24/20</f>
-        <v>1.2</v>
-      </c>
-      <c r="C7" s="2">
-        <v>0.2</v>
-      </c>
-      <c r="D7" s="1">
-        <f>0.3/12*1000</f>
-        <v>24.999999999999996</v>
-      </c>
-      <c r="E7" s="2">
-        <v>2200</v>
-      </c>
-      <c r="F7">
-        <v>12000</v>
-      </c>
-      <c r="G7">
-        <v>1600</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="H8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9">
-        <f>6/(1.8^2)</f>
-        <v>1.8518518518518516</v>
-      </c>
-      <c r="C9">
-        <f>C5</f>
-        <v>0.128</v>
-      </c>
-      <c r="D9">
-        <f>0.3/1.8*1000</f>
-        <v>166.66666666666666</v>
-      </c>
-      <c r="E9">
-        <v>57</v>
-      </c>
-      <c r="F9">
-        <v>12000</v>
-      </c>
-      <c r="G9">
-        <v>1600</v>
-      </c>
-      <c r="H9" t="s">
-        <v>16</v>
-      </c>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="C7" s="2"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="2"/>
+      <c r="H7" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H7" r:id="rId1" xr:uid="{A8D4DA74-31D2-4D8D-ABB1-19E58F228A4D}"/>
+    <hyperlink ref="J2" r:id="rId1" xr:uid="{48B40E40-3234-4F7D-B3C4-E06BBF351AFC}"/>
+    <hyperlink ref="J3" r:id="rId2" xr:uid="{DD13CAC7-322E-410C-AD32-41E9FE412601}"/>
+    <hyperlink ref="J4" r:id="rId3" xr:uid="{3CC7D07A-0A2F-4CC2-865A-61819A4FF125}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="256" orientation="landscape" horizontalDpi="500" verticalDpi="500" copies="0" r:id="rId2"/>
+  <pageSetup paperSize="256" orientation="landscape" horizontalDpi="500" verticalDpi="500" copies="0" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ktune GUI will export tuned PID values, saving and loading functions, testing spring damper system
</commit_message>
<xml_diff>
--- a/software/matlab/motors.xlsx
+++ b/software/matlab/motors.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flipa\OneDrive - UBC\University\Course Materials\3rd year\ELEC 391\robot-piano-player\software\matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EA4DC98-DF3F-4C99-9FD7-1732EF2C9F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC2F8D29-0C15-4622-A678-D661E70DDAA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A00A6A0-CC9E-4CD9-B7FE-C8C2B9679AFB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>Motor</t>
   </si>
@@ -84,6 +84,15 @@
   </si>
   <si>
     <t>https://ca.robotshop.com/products/e-s-motor-60d-planetary-gear-motor-with-high-torque-and-compact-size-24v-1660rpm?qd=650ebc719b16f099bd5f5e09cc852c24</t>
+  </si>
+  <si>
+    <t>Stall Torque (Nm)</t>
+  </si>
+  <si>
+    <t>Polulu37D_64CPR</t>
+  </si>
+  <si>
+    <t>https://www.pololu.com/product/4690/specs</t>
   </si>
 </sst>
 </file>
@@ -117,22 +126,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <u/>
-      <sz val="10"/>
+      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -172,19 +181,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -524,159 +537,221 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176A19DF-95F4-4146-B9C9-3E67B92D887F}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.453125" customWidth="1"/>
-    <col min="2" max="2" width="11.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.54296875" customWidth="1"/>
     <col min="6" max="6" width="11.81640625" customWidth="1"/>
-    <col min="7" max="9" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.08984375" customWidth="1"/>
+    <col min="10" max="10" width="8.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="40" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:12" ht="43" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="6" t="s">
         <v>9</v>
       </c>
+      <c r="L1" s="5"/>
     </row>
-    <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:12" ht="29" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="4">
+        <f>24/J2</f>
         <v>1.2</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="7">
         <v>0.2</v>
       </c>
-      <c r="D2" s="5">
-        <v>25</v>
-      </c>
-      <c r="E2" s="6">
+      <c r="D2" s="4">
+        <f>I2/J2*1000</f>
+        <v>250</v>
+      </c>
+      <c r="E2" s="7">
         <v>1471.4963</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="4">
         <v>12000</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="4">
         <v>1600</v>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="4">
         <v>3.6</v>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="4">
+        <v>5</v>
+      </c>
+      <c r="J2" s="4">
         <v>20</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="K2" s="9" t="s">
         <v>7</v>
       </c>
+      <c r="L2" s="5"/>
     </row>
-    <row r="3" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="5">
-        <v>3.692307692</v>
-      </c>
-      <c r="C3" s="6">
+      <c r="B3" s="4">
+        <f>24/J3</f>
+        <v>0.64864864864864868</v>
+      </c>
+      <c r="C3" s="7">
         <v>0.1</v>
       </c>
-      <c r="D3" s="5">
-        <v>12.06972</v>
-      </c>
-      <c r="E3" s="6">
+      <c r="D3" s="4">
+        <f>I3/J3*1000</f>
+        <v>7.9540540540540547</v>
+      </c>
+      <c r="E3" s="7">
         <v>192.24468999999999</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="4">
         <v>16000</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="4">
         <v>500</v>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="4">
         <v>1</v>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="6">
+        <v>0.29430000000000001</v>
+      </c>
+      <c r="J3" s="4">
         <v>37</v>
       </c>
-      <c r="J3" s="7" t="s">
+      <c r="K3" s="9" t="s">
         <v>8</v>
       </c>
+      <c r="L3" s="5"/>
     </row>
-    <row r="4" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="4">
+        <f>24/J4</f>
         <v>1.6</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="7">
         <v>0.1</v>
       </c>
-      <c r="D4" s="5">
-        <v>66.666666669999998</v>
-      </c>
-      <c r="E4" s="6">
+      <c r="D4" s="4">
+        <f>I4/J4*1000</f>
+        <v>80</v>
+      </c>
+      <c r="E4" s="7">
         <v>1434.6000899999999</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="4">
         <v>6000</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <v>400</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="4">
         <v>3.6</v>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="4">
+        <v>1.2</v>
+      </c>
+      <c r="J4" s="4">
         <v>15</v>
       </c>
-      <c r="J4" s="7" t="s">
+      <c r="K4" s="9" t="s">
         <v>15</v>
       </c>
+      <c r="L4" s="5"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="29" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4">
+        <v>8</v>
+      </c>
+      <c r="C5" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="D5" s="4">
+        <v>18.333333329999999</v>
+      </c>
+      <c r="E5" s="7">
+        <v>82.324640000000002</v>
+      </c>
+      <c r="F5" s="4">
+        <v>10000</v>
+      </c>
+      <c r="G5" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="H5" s="4">
+        <v>10</v>
+      </c>
+      <c r="I5" s="4">
+        <v>5.3955000000000003E-2</v>
+      </c>
+      <c r="J5" s="4">
+        <v>3</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="L5" s="5"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="C7" s="2"/>
       <c r="D7" s="1"/>
       <c r="E7" s="2"/>
       <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J2" r:id="rId1" xr:uid="{48B40E40-3234-4F7D-B3C4-E06BBF351AFC}"/>
-    <hyperlink ref="J3" r:id="rId2" xr:uid="{DD13CAC7-322E-410C-AD32-41E9FE412601}"/>
-    <hyperlink ref="J4" r:id="rId3" xr:uid="{3CC7D07A-0A2F-4CC2-865A-61819A4FF125}"/>
+    <hyperlink ref="K2" r:id="rId1" xr:uid="{48B40E40-3234-4F7D-B3C4-E06BBF351AFC}"/>
+    <hyperlink ref="K3" r:id="rId2" xr:uid="{DD13CAC7-322E-410C-AD32-41E9FE412601}"/>
+    <hyperlink ref="K4" r:id="rId3" xr:uid="{3CC7D07A-0A2F-4CC2-865A-61819A4FF125}"/>
+    <hyperlink ref="K5" r:id="rId4" xr:uid="{2137D88B-8585-4EEF-BDA7-EECD2C901E68}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="256" orientation="landscape" horizontalDpi="500" verticalDpi="500" copies="0" r:id="rId4"/>
+  <pageSetup paperSize="256" orientation="landscape" horizontalDpi="500" verticalDpi="500" copies="0" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mech step files, PID tuning for Polulu37D
</commit_message>
<xml_diff>
--- a/software/matlab/motors.xlsx
+++ b/software/matlab/motors.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flipa\OneDrive - UBC\University\Course Materials\3rd year\ELEC 391\robot-piano-player\software\matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA7E0F18-FB0A-484A-9300-0AD043F44FE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1E7B43-EB1C-41D8-A473-8F22DF4B5433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A00A6A0-CC9E-4CD9-B7FE-C8C2B9679AFB}"/>
   </bookViews>
@@ -587,7 +587,7 @@
       </c>
       <c r="L1" s="5"/>
     </row>
-    <row r="2" spans="1:12" ht="29" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
@@ -600,7 +600,7 @@
       </c>
       <c r="D2" s="4">
         <f>I2/J2*1000</f>
-        <v>250</v>
+        <v>17.57</v>
       </c>
       <c r="E2" s="7">
         <v>1471.4963</v>
@@ -615,7 +615,7 @@
         <v>3.6</v>
       </c>
       <c r="I2" s="4">
-        <v>5</v>
+        <v>0.35139999999999999</v>
       </c>
       <c r="J2" s="4">
         <v>20</v>
@@ -712,7 +712,8 @@
         <v>0.1</v>
       </c>
       <c r="D5" s="4">
-        <v>18.333333329999999</v>
+        <f>I5/J5*1000</f>
+        <v>17.984999999999999</v>
       </c>
       <c r="E5" s="7">
         <v>82.324640000000002</v>

</xml_diff>

<commit_message>
Tuned PID values baesd on inertia test values
</commit_message>
<xml_diff>
--- a/software/matlab/motors.xlsx
+++ b/software/matlab/motors.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\flipa\OneDrive - UBC\University\Course Materials\3rd year\ELEC 391\robot-piano-player\software\matlab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1E7B43-EB1C-41D8-A473-8F22DF4B5433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58F79800-8C06-439B-A482-9E30DEC9F956}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A00A6A0-CC9E-4CD9-B7FE-C8C2B9679AFB}"/>
   </bookViews>
@@ -701,7 +701,7 @@
       </c>
       <c r="L4" s="5"/>
     </row>
-    <row r="5" spans="1:12" ht="29" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="6" t="s">
         <v>17</v>
       </c>
@@ -716,13 +716,14 @@
         <v>17.984999999999999</v>
       </c>
       <c r="E5" s="7">
-        <v>82.324640000000002</v>
+        <v>20</v>
       </c>
       <c r="F5" s="4">
         <v>10000</v>
       </c>
       <c r="G5" s="4">
-        <v>0.1</v>
+        <f>0.07*1000</f>
+        <v>70</v>
       </c>
       <c r="H5" s="4">
         <v>10</v>

</xml_diff>